<commit_message>
adjust: add attr and metric for high level dim modeling and add staging database
</commit_message>
<xml_diff>
--- a/Docs/High-Level-Dimensional-Modeling-Workbook.xlsx
+++ b/Docs/High-Level-Dimensional-Modeling-Workbook.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HCMUTE\HCMUTE_HK6\DataWarehouse\final\airline-dwh\Docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21600" windowHeight="8130" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="8130" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="5" r:id="rId1"/>
@@ -15,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Issues List'!$A$1:$I$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +43,7 @@
     <author>mafudge</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0">
+    <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -55,7 +60,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A2" authorId="0">
+    <comment ref="A2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -67,7 +72,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B2" authorId="0">
+    <comment ref="B2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -79,7 +84,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C2" authorId="0">
+    <comment ref="C2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -91,7 +96,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D2" authorId="0">
+    <comment ref="D2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -103,7 +108,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E2" authorId="0">
+    <comment ref="E2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -126,7 +131,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F2" authorId="0">
+    <comment ref="F2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -148,7 +153,7 @@
     <author>mafudge</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0">
+    <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -163,7 +168,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A2" authorId="0">
+    <comment ref="A2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -175,7 +180,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B2" authorId="0">
+    <comment ref="B2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -187,7 +192,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C2" authorId="0">
+    <comment ref="C2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -199,7 +204,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D2" authorId="0">
+    <comment ref="D2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -211,7 +216,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E2" authorId="0">
+    <comment ref="E2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -234,7 +239,7 @@
     <author>mafudge</author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0">
+    <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -246,7 +251,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0">
+    <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -258,7 +263,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -270,7 +275,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -282,7 +287,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -294,7 +299,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -307,7 +312,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -319,7 +324,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -337,7 +342,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="108">
   <si>
     <t>Instructions!</t>
   </si>
@@ -377,9 +382,6 @@
     <t>Aircraft</t>
   </si>
   <si>
-    <t>Dim6</t>
-  </si>
-  <si>
     <t>Dim7</t>
   </si>
   <si>
@@ -501,24 +503,202 @@
   <si>
     <t>Date
 Closed</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+  <si>
+    <t>800, 1200, 2500</t>
+  </si>
+  <si>
+    <t>Arr_Delay_Mins</t>
+  </si>
+  <si>
+    <t>15, 30, 120</t>
+  </si>
+  <si>
+    <t>Estimated_Financial_Loss_USD</t>
+  </si>
+  <si>
+    <t>1113.60, 2227.20</t>
+  </si>
+  <si>
+    <t>Daily_Flight_Count</t>
+  </si>
+  <si>
+    <t>1, 4, 8</t>
+  </si>
+  <si>
+    <t>Tech_Incident_Count</t>
+  </si>
+  <si>
+    <t>0, 1, 2</t>
+  </si>
+  <si>
+    <t>Cumulative_Flight_Hours</t>
+  </si>
+  <si>
+    <t>500.5, 2400.0</t>
+  </si>
+  <si>
+    <t>Actual_Turnaround_Mins</t>
+  </si>
+  <si>
+    <t>45, 65, 120</t>
+  </si>
+  <si>
+    <t>Turnaround_Variance_Mins</t>
+  </si>
+  <si>
+    <t>-5, 10, 30</t>
+  </si>
+  <si>
+    <t>Dim_Date</t>
+  </si>
+  <si>
+    <t>CalendarQuarter</t>
+  </si>
+  <si>
+    <t>1, 2</t>
+  </si>
+  <si>
+    <t>IsWeekend</t>
+  </si>
+  <si>
+    <t>0, 1</t>
+  </si>
+  <si>
+    <t>Dim_Time</t>
+  </si>
+  <si>
+    <t>TimePeriod</t>
+  </si>
+  <si>
+    <t>Morning, Night</t>
+  </si>
+  <si>
+    <t>Dim_Airport</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Atlanta, Chicago, Dallas</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>GA, IL, TX</t>
+  </si>
+  <si>
+    <t>Dim_Airline</t>
+  </si>
+  <si>
+    <t>AirlineName</t>
+  </si>
+  <si>
+    <t>Delta Air Lines, United Airlines</t>
+  </si>
+  <si>
+    <t>Dim_Aircraft</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>BOEING, AIRBUS</t>
+  </si>
+  <si>
+    <t>AircraftAgeBand</t>
+  </si>
+  <si>
+    <t>&lt;5 yrs, &gt;15 yrs</t>
+  </si>
+  <si>
+    <t>Is_Active</t>
+  </si>
+  <si>
+    <t>Audit</t>
+  </si>
+  <si>
+    <t>Flight distance measured in statute miles.</t>
+  </si>
+  <si>
+    <t>Arrival delay in minutes (positive values indicate a delay).</t>
+  </si>
+  <si>
+    <t>Estimated financial impact of delay (Arrival Delay * $74.24).</t>
+  </si>
+  <si>
+    <t>Total number of flight segments completed by an aircraft per day.</t>
+  </si>
+  <si>
+    <t>Number of technical incidents (Carrier Delay &gt; 0) per day.</t>
+  </si>
+  <si>
+    <t>Total accumulated flight hours for an aircraft as of the current date.</t>
+  </si>
+  <si>
+    <t>Actual duration spent on the ground between two consecutive flights.</t>
+  </si>
+  <si>
+    <t>Difference between actual turnaround time and planned schedule.</t>
+  </si>
+  <si>
+    <t>Calendar quarter of the year (1, 2, 3, 4).</t>
+  </si>
+  <si>
+    <t>Flag indicating weekend (1 = Sat/Sun, 0 = Weekday).</t>
+  </si>
+  <si>
+    <t>Time of day classification (Morning, Afternoon, Evening, Night).</t>
+  </si>
+  <si>
+    <t>Name of the city where the airport is located.</t>
+  </si>
+  <si>
+    <t>Two-letter state code.</t>
+  </si>
+  <si>
+    <t>Full legal name of the airline carrier.</t>
+  </si>
+  <si>
+    <t>Name of the aircraft manufacturer.</t>
+  </si>
+  <si>
+    <t>Derived aircraft age group (&lt;5 yrs, 5-15 yrs, &gt;15 yrs).</t>
+  </si>
+  <si>
+    <t>SCD Type 2 status flag (1 = Current active record, 0 = Historical record).</t>
+  </si>
+  <si>
+    <t>Dim_Audit</t>
+  </si>
+  <si>
+    <t>ETL_Package_Name</t>
+  </si>
+  <si>
+    <t>Name of the SSIS package that loaded the record</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -539,157 +719,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
@@ -700,8 +729,16 @@
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="37">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -710,7 +747,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.79995117038483843"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -722,204 +759,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.79995117038483843"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.79995117038483843"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -942,253 +793,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1196,88 +805,51 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -1286,7 +858,7 @@
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5562599" cy="4819650"/>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1"/>
         <xdr:cNvSpPr txBox="1"/>
@@ -1342,7 +914,6 @@
             <a:rPr lang="en-US" sz="2000" b="1" baseline="0"/>
             <a:t> Modeling Worksheet</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="2000" b="1" baseline="0"/>
         </a:p>
         <a:p>
           <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
@@ -1381,10 +952,6 @@
             </a:rPr>
             <a:t>using the notes from the design session.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:endParaRPr lang="en-US" sz="1000" baseline="0">
@@ -1400,10 +967,6 @@
             </a:rPr>
             <a:t>What you will need:</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="1" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1426,10 +989,6 @@
             </a:rPr>
             <a:t>   and / or </a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1439,10 +998,6 @@
             </a:rPr>
             <a:t> - Enterprise bus matrix of processes and dimensions.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:endParaRPr lang="en-US" sz="1000" baseline="0">
@@ -1458,10 +1013,6 @@
             </a:rPr>
             <a:t>Procedure </a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="1" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1512,10 +1063,6 @@
             </a:rPr>
             <a:t>(from your requirements)</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1539,10 +1086,6 @@
             </a:rPr>
             <a:t> (type &amp; granularity)</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1566,10 +1109,6 @@
             </a:rPr>
             <a:t>used by this business process</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1593,10 +1132,6 @@
             </a:rPr>
             <a:t>from the business process </a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1620,10 +1155,6 @@
             </a:rPr>
             <a:t> section:</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1646,10 +1177,6 @@
             </a:rPr>
             <a:t>      dimension, keeping in mind all of the business processes.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1686,10 +1213,6 @@
             </a:rPr>
             <a:t>      you have them. </a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1699,10 +1222,6 @@
             </a:rPr>
             <a:t>   3) Do the same for each fact table, explain derived facts.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -1739,10 +1258,6 @@
             </a:rPr>
             <a:t>tab so that you remember to address them at a later time.</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
-            <a:latin typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-            <a:cs typeface="Consolas" panose="020B0609020204030204" pitchFamily="49" charset="0"/>
-          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:endParaRPr lang="en-US" sz="1000" b="0" baseline="0">
@@ -2041,49 +1556,49 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor theme="3" tint="0.799981688894314"/>
+    <tabColor theme="3" tint="0.79995117038483843"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9.17699115044248" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" width="9.17699115044248" style="13"/>
+    <col min="1" max="16384" width="9.140625" style="13"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor theme="5" tint="0.599993896298105"/>
+    <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:S14"/>
-  <sheetFormatPr defaultColWidth="9.17699115044248" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.3716814159292" style="7" customWidth="1"/>
-    <col min="2" max="2" width="25.1592920353982" style="7" customWidth="1"/>
-    <col min="3" max="3" width="19.5132743362832" style="7" customWidth="1"/>
-    <col min="4" max="4" width="28.3451327433628" style="7" customWidth="1"/>
-    <col min="5" max="5" width="70.6283185840708" style="7" customWidth="1"/>
-    <col min="6" max="19" width="3.72566371681416" style="7" customWidth="1"/>
-    <col min="20" max="16384" width="9.17699115044248" style="7"/>
+    <col min="1" max="1" width="22.42578125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" style="7" customWidth="1"/>
+    <col min="4" max="4" width="45.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="80.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="19" width="3.7109375" style="7" customWidth="1"/>
+    <col min="20" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:19">
+    <row r="1" spans="1:19" ht="14.25" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="66.75" customHeight="1" spans="1:19">
+    <row r="2" spans="1:19" ht="66.75" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
@@ -2114,66 +1629,68 @@
       <c r="J2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="K2" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="M2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="N2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="O2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="P2" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="Q2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="R2" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="S2" s="10" t="s">
         <v>18</v>
-      </c>
-      <c r="S2" s="10" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>23</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="11" t="s">
-        <v>25</v>
-      </c>
       <c r="G3" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3" s="11"/>
+        <v>24</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>24</v>
+      </c>
       <c r="L3" s="11"/>
       <c r="M3" s="11"/>
       <c r="N3" s="11"/>
@@ -2185,32 +1702,34 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
         <v>26</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>27</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>28</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" t="s">
-        <v>30</v>
-      </c>
       <c r="F4" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>
       <c r="I4" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" s="11"/>
+        <v>24</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>24</v>
+      </c>
       <c r="L4" s="11"/>
       <c r="M4" s="11"/>
       <c r="N4" s="11"/>
@@ -2222,36 +1741,38 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
         <v>31</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>33</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>34</v>
       </c>
-      <c r="E5" t="s">
-        <v>35</v>
-      </c>
       <c r="F5" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="K5" s="11"/>
+        <v>24</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>24</v>
+      </c>
       <c r="L5" s="11"/>
       <c r="M5" s="11"/>
       <c r="N5" s="11"/>
@@ -2452,26 +1973,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor theme="9" tint="0.399975585192419"/>
+    <tabColor theme="9" tint="0.39994506668294322"/>
   </sheetPr>
   <dimension ref="A1:E64"/>
-  <sheetFormatPr defaultColWidth="9.17699115044248" defaultRowHeight="14.25" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="33.8141592920354" style="4" customWidth="1"/>
-    <col min="2" max="2" width="31.7256637168142" style="4" customWidth="1"/>
-    <col min="3" max="3" width="40.5398230088496" style="4" customWidth="1"/>
-    <col min="4" max="4" width="15.8141592920354" style="4" customWidth="1"/>
-    <col min="5" max="5" width="23.2654867256637" style="4" customWidth="1"/>
-    <col min="6" max="16384" width="9.17699115044248" style="4"/>
+    <col min="1" max="1" width="33.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="64.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" style="4" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2479,148 +1999,290 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="28.5" spans="1:5">
+    <row r="2" spans="1:5" ht="30">
       <c r="A2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="A3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
+      <c r="E4" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
+      <c r="A6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+      <c r="A7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>92</v>
+      </c>
       <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
+      <c r="A8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+      <c r="A9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>94</v>
+      </c>
       <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
+      <c r="E9" s="3" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
+      <c r="A10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
+      <c r="E10" s="3" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+      <c r="A11" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>107</v>
+      </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+      <c r="A12" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
+      <c r="A13" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>97</v>
+      </c>
       <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
+      <c r="E13" s="3" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
+      <c r="A14" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>98</v>
+      </c>
       <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
+      <c r="A15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>99</v>
+      </c>
       <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="E15" s="3" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+      <c r="A16" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>100</v>
+      </c>
       <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
+      <c r="E16" s="3" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+      <c r="A17" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>101</v>
+      </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>102</v>
+      </c>
       <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
+      <c r="E18" s="3" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+      <c r="A19" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>103</v>
+      </c>
       <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
+      <c r="E19" s="3" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
+      <c r="A20" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>104</v>
+      </c>
       <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
+      <c r="E20" s="3" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="3"/>
@@ -2932,58 +2594,58 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor theme="7" tint="0.799981688894314"/>
+    <tabColor theme="7" tint="0.79995117038483843"/>
   </sheetPr>
   <dimension ref="A1:I253"/>
-  <sheetFormatPr defaultColWidth="9.17699115044248" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.26548672566372" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.45132743362832" style="1" customWidth="1"/>
-    <col min="3" max="3" width="41.2654867256637" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1769911504425" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5398230088496" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5398230088496" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.72566371681416" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.8141592920354" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.26548672566372" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.17699115044248" style="1"/>
+    <col min="1" max="1" width="9.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.5" spans="1:9">
+    <row r="1" spans="1:9" ht="30">
       <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -5759,11 +5421,8 @@
       <c r="I253" s="3"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I1" etc:filterBottomFollowUsedRange="0">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>